<commit_message>
feat: complete sports center workflow updates
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Reba6d9e5f04649f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rb151dda1266f4e53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rfb1ebc0a14cc405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R6e87df74b7264faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R5e4e15cdf6d14a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R8a7660485af54bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Ra3fab6ec6e6941a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rd0535c30ca664878"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -173,7 +173,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -248,6 +248,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -320,8 +323,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Version1TaskTable" displayName="Version1TaskTable" ref="A4:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:J15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Version1TaskTable" displayName="Version1TaskTable" ref="A4:J16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J16"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Source requirement IDs"/>
@@ -339,8 +342,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProductionTaskTable" displayName="ProductionTaskTable" ref="A4:J14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:J14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProductionTaskTable" displayName="ProductionTaskTable" ref="A4:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J15"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Source requirement IDs"/>
@@ -838,13 +841,13 @@
         <x:v>FR-009</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Training progress</x:v>
+        <x:v>Training plans and progress</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Coach, Member</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
-        <x:v>Coach records training results, plans and comments for assigned Members; Member views their own records.</x:v>
+        <x:v>Coach creates and maintains multi-exercise personal training plans for assigned Members, then records results and comments. Member views only their own plans and results.</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
         <x:v>Must</x:v>
@@ -853,10 +856,10 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
-        <x:v>Each Member has one active primary Coach at a time. Coach can edit only assigned Members; Member cannot edit coach records.</x:v>
+        <x:v>An MVP plan stores its name, goal, start and end dates plus one or more exercises. Each exercise has a name, sets, repetitions or duration, rest time and an optional note. Coach can edit only assigned Members; Member cannot edit Coach records.</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -896,7 +899,7 @@
         <x:v>Manager</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>Manager views basic member, class attendance and payment-status revenue summaries.</x:v>
+        <x:v>Manager dashboard summarizes center-wide revenue, members, classes, bookings and attendance for a selected day, week, month, quarter or year. It compares each KPI with the immediately preceding equivalent period and provides role-scoped operational summaries for other users.</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
         <x:v>Should</x:v>
@@ -905,10 +908,10 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G15" s="18" t="str">
-        <x:v>Revenue uses only successful payments and groups payment states separately; date filtering uses successful payment time.</x:v>
+        <x:v>Changing the period refreshes every dashboard KPI and trend. Each comparison uses the immediately preceding period of equal duration. Revenue uses paid_at for confirmed cash payments only; pending payments and memberships expiring within 7 days remain visible as actionable alerts.</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -1198,7 +1201,7 @@
         <x:v>Assigned classes and students</x:v>
       </x:c>
       <x:c r="C31" s="26" t="str">
-        <x:v>Plans, results, comments</x:v>
+        <x:v>Plans, exercises, results, comments</x:v>
       </x:c>
       <x:c r="D31" s="26" t="str">
         <x:v>Own assigned records</x:v>
@@ -1460,9 +1463,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a2e0fc8c8954aec"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a1cbd59ce2f4423"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54de02aaff3748ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180a7a14014e4910"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf55fdadedfd4b65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb482a17b8474dbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1790,13 +1793,13 @@
         <x:v>FR-009</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>Progress</x:v>
+        <x:v>Training plans</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Coach records plan, result and comment for assigned Member.</x:v>
+        <x:v>Coach creates multi-exercise personal plans and records a result for an assigned Member.</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>Basic training progress</x:v>
+        <x:v>Plan details plus one or more exercise items: name, sets, repetitions or duration, rest time and optional note. One general result and Coach comment per recorded date.</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
         <x:v>Backend + Frontend</x:v>
@@ -1808,10 +1811,10 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
-        <x:v>Member can view but cannot alter Coach records.</x:v>
+        <x:v>A plan cannot be saved without an exercise. Coach can add, edit, remove and order exercises for an assigned Member. Member can view the plan and results but cannot alter Coach records.</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
@@ -1857,10 +1860,10 @@
         <x:v>Dashboard</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>Manager sees basic members, bookings, attendance and payment-status revenue.</x:v>
+        <x:v>Manager can review center performance and compare it with the prior equivalent period.</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>Date filter based on successful payment timestamp; separate payment statuses</x:v>
+        <x:v>Period selector: day, week, month, quarter and year; four KPI cards, revenue trend and actionable alerts. Receptionist, Coach and Member receive only role-scoped summaries.</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
         <x:v>Frontend + QA</x:v>
@@ -1872,10 +1875,10 @@
         <x:v>Should</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
-        <x:v>Revenue sums successful payments only. Pending and failed payments remain visible as separate operational measures.</x:v>
+        <x:v>Changing the period updates all metrics. Revenue includes confirmed cash payments only; each KPI shows the comparison with the immediately preceding equivalent period. Pending cash receipts and memberships expiring within 7 days open their related lists.</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -1917,7 +1920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33bed4630d724e1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb88c1a0910a4271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2365,6 +2368,38 @@
         <x:v>Planned</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="96" customHeight="1">
+      <x:c r="A16" s="30" t="str">
+        <x:v>V1-012</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>FR-009</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>Training plans</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Coach organizes a plan into workout sessions and tracks each session's completion.</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Ordered sessions with title and optional scheduled date. Each session contains exercises. Coach records completed or skipped status and a session comment.</x:v>
+      </x:c>
+      <x:c r="F16" s="30" t="str">
+        <x:v>Backend + Frontend</x:v>
+      </x:c>
+      <x:c r="G16" s="30" t="str">
+        <x:v>MVP training plans</x:v>
+      </x:c>
+      <x:c r="H16" s="30" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="I16" s="30" t="str">
+        <x:v>A Coach can reorder sessions and exercises. Completing or skipping a session keeps its timestamp and Coach comment. Member sees only their own session status and feedback.</x:v>
+      </x:c>
+      <x:c r="J16" s="30" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -2372,7 +2407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cab8705f3f7437d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75fd6acbae14b31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2788,6 +2823,38 @@
         <x:v>Planned</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="96" customHeight="1">
+      <x:c r="A15" s="30" t="str">
+        <x:v>PROD-011</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>FR-009, NFR-004</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>Training analytics</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="str">
+        <x:v>System tracks progressive training performance and plan adjustments over time.</x:v>
+      </x:c>
+      <x:c r="E15" s="30" t="str">
+        <x:v>Actual load, achieved sets/repetitions or duration, optional effort rating, progress charts and plan version history.</x:v>
+      </x:c>
+      <x:c r="F15" s="30" t="str">
+        <x:v>Backend + Frontend + QA</x:v>
+      </x:c>
+      <x:c r="G15" s="30" t="str">
+        <x:v>Version 1 training sessions</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="I15" s="30" t="str">
+        <x:v>Trend charts use recorded performance data. Each plan adjustment is traceable to a version and timestamp. Coach scope and Member privacy remain enforced.</x:v>
+      </x:c>
+      <x:c r="J15" s="30" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -2795,7 +2862,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18b7d2bc0e3d44d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb22edd8f603d4cfb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add version 1 comparison gates
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R5e4e15cdf6d14a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R8a7660485af54bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Ra3fab6ec6e6941a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rd0535c30ca664878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rf0e252e5e61f4c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rca7e808131c44eb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R6fc3ffa5a7c0497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R01c9aebf2d8744ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,8 +44,14 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -62,8 +68,18 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173F68"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB9E0F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -169,11 +185,25 @@
         <x:color rgb="FFE0E6EB"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF58BCEB"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF58BCEB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF58BCEB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF58BCEB"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -250,6 +280,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1463,9 +1514,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180a7a14014e4910"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf55fdadedfd4b65"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb482a17b8474dbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670dac7c5a2d481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc62c8777c149d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b372ae99e084d63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1971,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb88c1a0910a4271"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc16494a1d1e842fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1942,6 +1993,8 @@
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1960,7 +2013,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="str">
-        <x:v>Goal: make the system usable in daily operations at one real center. Tasks are derived from the requirement IDs in System Requirements.</x:v>
+        <x:v>Goal: make the system usable in daily operations at one real center. Compare each Version 1 item only after its MVP baseline and gate evidence are accepted.</x:v>
       </x:c>
       <x:c r="B2" s="10"/>
       <x:c r="C2" s="10"/>
@@ -2015,6 +2068,12 @@
       <x:c r="J4" s="8" t="str">
         <x:v>Status</x:v>
       </x:c>
+      <x:c r="K4" s="35" t="str">
+        <x:v>MVP baseline for comparison</x:v>
+      </x:c>
+      <x:c r="L4" s="35" t="str">
+        <x:v>V1 gate</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="10" t="str">
@@ -2047,6 +2106,12 @@
       <x:c r="J5" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K5" s="37" t="str">
+        <x:v>MVP-004: package entitlement, paid activation and expiry/grace state verified.</x:v>
+      </x:c>
+      <x:c r="L5" s="37" t="str">
+        <x:v>Start after MVP-004 and notification foundation are accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="10" t="str">
@@ -2079,6 +2144,12 @@
       <x:c r="J6" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K6" s="36" t="str">
+        <x:v>MVP-006: capacity, duplicate prevention and cancellation behavior verified.</x:v>
+      </x:c>
+      <x:c r="L6" s="36" t="str">
+        <x:v>Start after MVP-006 is accepted and promotion policy is approved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="10" t="str">
@@ -2111,6 +2182,12 @@
       <x:c r="J7" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K7" s="37" t="str">
+        <x:v>MVP-009: manual/simulated payment lifecycle and membership activation verified.</x:v>
+      </x:c>
+      <x:c r="L7" s="37" t="str">
+        <x:v>Start after MVP-009 is accepted; provider contract and reconciliation owner assigned.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="10" t="str">
@@ -2143,6 +2220,12 @@
       <x:c r="J8" s="10" t="str">
         <x:v>Rejected by policy</x:v>
       </x:c>
+      <x:c r="K8" s="36" t="str">
+        <x:v>Policy baseline: FR-014 remains out of scope.</x:v>
+      </x:c>
+      <x:c r="L8" s="36" t="str">
+        <x:v>Keep excluded; any reversal needs a separately approved policy.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="10" t="str">
@@ -2175,6 +2258,12 @@
       <x:c r="J9" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K9" s="37" t="str">
+        <x:v>MVP-004 and MVP-007: active entitlement plus attendance data are verified.</x:v>
+      </x:c>
+      <x:c r="L9" s="37" t="str">
+        <x:v>Start after tablet flow, device ownership and check-in audit test are accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="10" t="str">
@@ -2207,6 +2296,12 @@
       <x:c r="J10" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K10" s="36" t="str">
+        <x:v>Core role-scoped data and class/package events are verified.</x:v>
+      </x:c>
+      <x:c r="L10" s="36" t="str">
+        <x:v>Start after notification channels, preferences and delivery failure handling are agreed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="10" t="str">
@@ -2239,6 +2334,12 @@
       <x:c r="J11" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K11" s="37" t="str">
+        <x:v>MVP-002: authorized-role access is verified.</x:v>
+      </x:c>
+      <x:c r="L11" s="37" t="str">
+        <x:v>Start after authorization regression suite is accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="10" t="str">
@@ -2271,6 +2372,12 @@
       <x:c r="J12" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K12" s="36" t="str">
+        <x:v>MVP-007, MVP-009 and MVP-010: attendance, paid revenue and dashboard metrics reconcile.</x:v>
+      </x:c>
+      <x:c r="L12" s="36" t="str">
+        <x:v>Start after report definitions, date/coach filters and export decision are accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="10" t="str">
@@ -2303,6 +2410,12 @@
       <x:c r="J13" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K13" s="37" t="str">
+        <x:v>MVP-001, MVP-002 and MVP-011: authentication, authorization and audit evidence are verified.</x:v>
+      </x:c>
+      <x:c r="L13" s="37" t="str">
+        <x:v>Start after rate-limit, privacy review and session-expiry tests are accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="10" t="str">
@@ -2335,6 +2448,12 @@
       <x:c r="J14" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K14" s="36" t="str">
+        <x:v>MVP-008 and V1-006: training context and notification foundations are verified.</x:v>
+      </x:c>
+      <x:c r="L14" s="36" t="str">
+        <x:v>Start only after AI policy, data-minimization review and Coach approval workflow are accepted.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="10" t="str">
@@ -2367,6 +2486,12 @@
       <x:c r="J15" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
+      <x:c r="K15" s="37" t="str">
+        <x:v>Database baseline and operational data ownership are verified.</x:v>
+      </x:c>
+      <x:c r="L15" s="37" t="str">
+        <x:v>Start after backup frequency, RPO/RTO targets and restore environment are approved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="96" customHeight="1">
       <x:c r="A16" s="30" t="str">
@@ -2398,6 +2523,12 @@
       </x:c>
       <x:c r="J16" s="30" t="str">
         <x:v>Proposed</x:v>
+      </x:c>
+      <x:c r="K16" s="36" t="str">
+        <x:v>MVP-008: multi-exercise plans and member/Coach scope are verified.</x:v>
+      </x:c>
+      <x:c r="L16" s="36" t="str">
+        <x:v>Start after session model, reorder behavior and completion audit tests are accepted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2407,7 +2538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75fd6acbae14b31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R515d696979084d71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2862,7 +2993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb22edd8f603d4cfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb36a165c0334ea8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "docs: add version 1 comparison gates"
This reverts commit 2af674ff2a3b89a9e71937fa94492d1cb3f8d13a.
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rf0e252e5e61f4c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rca7e808131c44eb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R6fc3ffa5a7c0497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R01c9aebf2d8744ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R5e4e15cdf6d14a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R8a7660485af54bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Ra3fab6ec6e6941a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rd0535c30ca664878"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,14 +44,8 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -68,18 +62,8 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF173F68"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFB9E0F1"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
-  <x:borders count="12">
+  <x:borders count="11">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -185,25 +169,11 @@
         <x:color rgb="FFE0E6EB"/>
       </x:top>
     </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FF58BCEB"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FF58BCEB"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FF58BCEB"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF58BCEB"/>
-      </x:bottom>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -280,27 +250,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1514,9 +1463,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670dac7c5a2d481a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc62c8777c149d8"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b372ae99e084d63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180a7a14014e4910"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf55fdadedfd4b65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb482a17b8474dbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1971,7 +1920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc16494a1d1e842fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb88c1a0910a4271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1993,8 +1942,6 @@
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2013,7 +1960,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="str">
-        <x:v>Goal: make the system usable in daily operations at one real center. Compare each Version 1 item only after its MVP baseline and gate evidence are accepted.</x:v>
+        <x:v>Goal: make the system usable in daily operations at one real center. Tasks are derived from the requirement IDs in System Requirements.</x:v>
       </x:c>
       <x:c r="B2" s="10"/>
       <x:c r="C2" s="10"/>
@@ -2068,12 +2015,6 @@
       <x:c r="J4" s="8" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="K4" s="35" t="str">
-        <x:v>MVP baseline for comparison</x:v>
-      </x:c>
-      <x:c r="L4" s="35" t="str">
-        <x:v>V1 gate</x:v>
-      </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="10" t="str">
@@ -2106,12 +2047,6 @@
       <x:c r="J5" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K5" s="37" t="str">
-        <x:v>MVP-004: package entitlement, paid activation and expiry/grace state verified.</x:v>
-      </x:c>
-      <x:c r="L5" s="37" t="str">
-        <x:v>Start after MVP-004 and notification foundation are accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="10" t="str">
@@ -2144,12 +2079,6 @@
       <x:c r="J6" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K6" s="36" t="str">
-        <x:v>MVP-006: capacity, duplicate prevention and cancellation behavior verified.</x:v>
-      </x:c>
-      <x:c r="L6" s="36" t="str">
-        <x:v>Start after MVP-006 is accepted and promotion policy is approved.</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="10" t="str">
@@ -2182,12 +2111,6 @@
       <x:c r="J7" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K7" s="37" t="str">
-        <x:v>MVP-009: manual/simulated payment lifecycle and membership activation verified.</x:v>
-      </x:c>
-      <x:c r="L7" s="37" t="str">
-        <x:v>Start after MVP-009 is accepted; provider contract and reconciliation owner assigned.</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="10" t="str">
@@ -2220,12 +2143,6 @@
       <x:c r="J8" s="10" t="str">
         <x:v>Rejected by policy</x:v>
       </x:c>
-      <x:c r="K8" s="36" t="str">
-        <x:v>Policy baseline: FR-014 remains out of scope.</x:v>
-      </x:c>
-      <x:c r="L8" s="36" t="str">
-        <x:v>Keep excluded; any reversal needs a separately approved policy.</x:v>
-      </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="10" t="str">
@@ -2258,12 +2175,6 @@
       <x:c r="J9" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K9" s="37" t="str">
-        <x:v>MVP-004 and MVP-007: active entitlement plus attendance data are verified.</x:v>
-      </x:c>
-      <x:c r="L9" s="37" t="str">
-        <x:v>Start after tablet flow, device ownership and check-in audit test are accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="10" t="str">
@@ -2296,12 +2207,6 @@
       <x:c r="J10" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K10" s="36" t="str">
-        <x:v>Core role-scoped data and class/package events are verified.</x:v>
-      </x:c>
-      <x:c r="L10" s="36" t="str">
-        <x:v>Start after notification channels, preferences and delivery failure handling are agreed.</x:v>
-      </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="10" t="str">
@@ -2334,12 +2239,6 @@
       <x:c r="J11" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K11" s="37" t="str">
-        <x:v>MVP-002: authorized-role access is verified.</x:v>
-      </x:c>
-      <x:c r="L11" s="37" t="str">
-        <x:v>Start after authorization regression suite is accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="10" t="str">
@@ -2372,12 +2271,6 @@
       <x:c r="J12" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K12" s="36" t="str">
-        <x:v>MVP-007, MVP-009 and MVP-010: attendance, paid revenue and dashboard metrics reconcile.</x:v>
-      </x:c>
-      <x:c r="L12" s="36" t="str">
-        <x:v>Start after report definitions, date/coach filters and export decision are accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="10" t="str">
@@ -2410,12 +2303,6 @@
       <x:c r="J13" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K13" s="37" t="str">
-        <x:v>MVP-001, MVP-002 and MVP-011: authentication, authorization and audit evidence are verified.</x:v>
-      </x:c>
-      <x:c r="L13" s="37" t="str">
-        <x:v>Start after rate-limit, privacy review and session-expiry tests are accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="10" t="str">
@@ -2448,12 +2335,6 @@
       <x:c r="J14" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K14" s="36" t="str">
-        <x:v>MVP-008 and V1-006: training context and notification foundations are verified.</x:v>
-      </x:c>
-      <x:c r="L14" s="36" t="str">
-        <x:v>Start only after AI policy, data-minimization review and Coach approval workflow are accepted.</x:v>
-      </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="10" t="str">
@@ -2486,12 +2367,6 @@
       <x:c r="J15" s="10" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="K15" s="37" t="str">
-        <x:v>Database baseline and operational data ownership are verified.</x:v>
-      </x:c>
-      <x:c r="L15" s="37" t="str">
-        <x:v>Start after backup frequency, RPO/RTO targets and restore environment are approved.</x:v>
-      </x:c>
     </x:row>
     <x:row r="16" ht="96" customHeight="1">
       <x:c r="A16" s="30" t="str">
@@ -2523,12 +2398,6 @@
       </x:c>
       <x:c r="J16" s="30" t="str">
         <x:v>Proposed</x:v>
-      </x:c>
-      <x:c r="K16" s="36" t="str">
-        <x:v>MVP-008: multi-exercise plans and member/Coach scope are verified.</x:v>
-      </x:c>
-      <x:c r="L16" s="36" t="str">
-        <x:v>Start after session model, reorder behavior and completion audit tests are accepted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2538,7 +2407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R515d696979084d71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75fd6acbae14b31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2993,7 +2862,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb36a165c0334ea8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb22edd8f603d4cfb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: scope receptionist check-in out
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R5e4e15cdf6d14a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R8a7660485af54bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Ra3fab6ec6e6941a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rd0535c30ca664878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Readebcbeb4294134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R4d5c72ed24b84a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R9893af5ff3d44e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R7753445650ab4f5f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -818,10 +818,10 @@
         <x:v>Attendance</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>Coach, Receptionist, Member</x:v>
+        <x:v>Coach, Member</x:v>
       </x:c>
       <x:c r="D12" s="18" t="str">
-        <x:v>Coach records class attendance; Receptionist performs facility check-in; Member sees own history.</x:v>
+        <x:v>Coach records class attendance; Member sees own history.</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
         <x:v>Must</x:v>
@@ -830,10 +830,10 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
-        <x:v>Class attendance and facility check-in are separate records. Coach corrections apply immediately with a reason and audit log.</x:v>
+        <x:v>Coach records present, absent or late for assigned classes. Corrections require a reason and create an audit log.</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -1463,9 +1463,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180a7a14014e4910"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf55fdadedfd4b65"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb482a17b8474dbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d9daa17dd0c4c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5c49bfbb6a4bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcc576f593bd48d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1779,10 +1779,10 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
-        <x:v>Only assigned Coach or authorized Receptionist records attendance. Coach corrections immediately retain actor, reason and previous/new values.</x:v>
+        <x:v>Only assigned Coach records attendance. Coach corrections retain actor, reason and previous/new values.</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -1920,7 +1920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb88c1a0910a4271"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1642595645fd4c00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2155,25 +2155,25 @@
         <x:v>Front desk</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>Receptionist performs facility check-in and supports member workflows.</x:v>
+        <x:v>Facility check-in is excluded by operating scope.</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>Tablet-friendly entrance flow separate from class attendance</x:v>
+        <x:v>No entrance check-in flow is required for Receptionist.</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>Product + Development</x:v>
+        <x:v>Business policy</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>Membership</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>Must</x:v>
+        <x:v>Out of scope</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
-        <x:v>Check-in validates active entitlement, records entrance timestamp and refuses pending-payment, expired or cancelled memberships.</x:v>
+        <x:v>The product provides no facility check-in flow. Class attendance remains Coach-led under FR-008.</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Rejected by policy</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
@@ -2407,7 +2407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75fd6acbae14b31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba581534019455a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2862,7 +2862,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb22edd8f603d4cfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c9e5cea43348ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(requirements): align MVP decisions
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Readebcbeb4294134"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R4d5c72ed24b84a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R9893af5ff3d44e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R7753445650ab4f5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R4c576fdc973641a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rc992933e8a30419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R7de3e8a408304887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R6241d1746d9b46de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -795,7 +795,7 @@
         <x:v>Member, Receptionist</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
-        <x:v>Member or Receptionist can register or cancel a class booking.</x:v>
+        <x:v>Member or Receptionist can register, cancel or join the waitlist for a class booking.</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
         <x:v>Must</x:v>
@@ -804,7 +804,7 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
-        <x:v>Expired members, duplicate bookings and full classes are rejected with a clear reason.</x:v>
+        <x:v>Expired members and duplicate bookings are rejected with a clear reason. When a class reaches capacity, the booking is waitlisted and is promoted in order when a confirmed place becomes available.</x:v>
       </x:c>
       <x:c r="H11" s="19" t="str">
         <x:v>Proposed</x:v>
@@ -847,7 +847,7 @@
         <x:v>Coach, Member</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
-        <x:v>Coach creates and maintains multi-exercise personal training plans for assigned Members, then records results and comments. Member views only their own plans and results.</x:v>
+        <x:v>Coach creates and maintains personal training plans for assigned Members, with optional exercises, then records results and comments. Member views only their own plans and results.</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
         <x:v>Must</x:v>
@@ -856,7 +856,7 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
-        <x:v>An MVP plan stores its name, goal, start and end dates plus one or more exercises. Each exercise has a name, sets, repetitions or duration, rest time and an optional note. Coach can edit only assigned Members; Member cannot edit Coach records.</x:v>
+        <x:v>An MVP plan stores its name, goal, start and end dates. Exercises are optional; each supplied exercise has a name, sets, repetitions or duration, rest time and an optional note. Coach can edit only assigned Members; Member cannot edit Coach records.</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
         <x:v>Updated</x:v>
@@ -1463,9 +1463,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d9daa17dd0c4c19"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5c49bfbb6a4bfc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcc576f593bd48d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e72a3ab82224aeb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R776c06118fa24cdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc047749eb643aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1486,7 +1486,7 @@
     <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25.6299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1590,7 +1590,7 @@
         <x:v>Correct credentials open the correct role landing page; invalid credentials are rejected.</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
@@ -1622,7 +1622,7 @@
         <x:v>Direct API access outside the role returns an authorization error.</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
@@ -1654,7 +1654,7 @@
         <x:v>Required fields validate and suspended staff cannot sign in.</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
@@ -1686,7 +1686,7 @@
         <x:v>Higher tiers inherit lower-tier entitlements. Only successful payment activates access; expired access is blocked after exactly 72 grace hours.</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
@@ -1718,7 +1718,7 @@
         <x:v>Invalid overlaps and missing required data are rejected.</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
@@ -1735,7 +1735,7 @@
         <x:v>Member or Receptionist can book and cancel classes.</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>No duplicate booking; capacity check</x:v>
+        <x:v>No duplicate booking; capacity check with ordered waitlist.</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
         <x:v>Backend + Frontend</x:v>
@@ -1747,10 +1747,10 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
-        <x:v>Full, expired and duplicate cases show clear errors.</x:v>
+        <x:v>Expired and duplicate cases show clear errors. A full class creates a waitlisted booking, and the earliest eligible waitlisted booking is promoted after a confirmed cancellation.</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
@@ -1782,7 +1782,7 @@
         <x:v>Only assigned Coach records attendance. Coach corrections retain actor, reason and previous/new values.</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>Updated</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -1796,10 +1796,10 @@
         <x:v>Training plans</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Coach creates multi-exercise personal plans and records a result for an assigned Member.</x:v>
+        <x:v>Coach creates a personal plan and records a result for an assigned Member.</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>Plan details plus one or more exercise items: name, sets, repetitions or duration, rest time and optional note. One general result and Coach comment per recorded date.</x:v>
+        <x:v>Plan details plus optional exercise items: name, sets, repetitions or duration, rest time and optional note. One general result and Coach comment per recorded date.</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
         <x:v>Backend + Frontend</x:v>
@@ -1811,10 +1811,10 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
-        <x:v>A plan cannot be saved without an exercise. Coach can add, edit, remove and order exercises for an assigned Member. Member can view the plan and results but cannot alter Coach records.</x:v>
+        <x:v>A plan can be saved with or without exercises. When exercises are included, Coach can add, edit, remove and order them for an assigned Member. Member can view the plan and results but cannot alter Coach records.</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Updated</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
@@ -1846,7 +1846,7 @@
         <x:v>A successful transaction includes amount, method, payer, membership and paid timestamp, then activates the membership. Pending/failed payment never activates access.</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
@@ -1878,7 +1878,7 @@
         <x:v>Changing the period updates all metrics. Revenue includes confirmed cash payments only; each KPI shows the comparison with the immediately preceding equivalent period. Pending cash receipts and memberships expiring within 7 days open their related lists.</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>Updated</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -1910,7 +1910,7 @@
         <x:v>Log includes actor, action, timestamp and target record.</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented - static verified</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1920,7 +1920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1642595645fd4c00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3b62b24fc6144d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2059,10 +2059,10 @@
         <x:v>Bookings</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>The system supports waitlists and cancellation rules.</x:v>
+        <x:v>The system refines waitlist notifications and cancellation rules.</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
-        <x:v>Capacity and cutoff policy</x:v>
+        <x:v>Notification timing and cancellation cutoff policy.</x:v>
       </x:c>
       <x:c r="F6" s="11" t="str">
         <x:v>Backend + Frontend</x:v>
@@ -2074,7 +2074,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
-        <x:v>Eligible waitlisted users are promoted according to a defined rule.</x:v>
+        <x:v>Waitlisted users receive clear status and promotion notifications. Cancellation rules are applied according to the defined cutoff policy.</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
         <x:v>Planned</x:v>
@@ -2407,7 +2407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba581534019455a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce9058c1b8846f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2862,7 +2862,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c9e5cea43348ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890ae0d2473f48f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(api): align version 1 delivery contracts
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R4c576fdc973641a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rc992933e8a30419e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R7de3e8a408304887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R6241d1746d9b46de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R51ef286399a64523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R7c6fca849c3648b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rbbfea0165c25438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R1f100769d17f4c78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1463,9 +1463,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e72a3ab82224aeb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R776c06118fa24cdd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc047749eb643aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c426c206d874e83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2394fb5ba95414b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb9a6ed3716249b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3b62b24fc6144d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb3f01d9e2c4923"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2091,10 +2091,10 @@
         <x:v>Payments</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>System supports real payment status and invoices.</x:v>
+        <x:v>System supports sandbox payment status and receipts before live go-live.</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>Gateway integration, receipt history</x:v>
+        <x:v>Sandbox gateway flows (VNPay, MoMo and ZaloPay), receipt history and signed callback simulation</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
         <x:v>Backend + Finance</x:v>
@@ -2106,10 +2106,10 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
-        <x:v>Success, failure, pending and refund states are handled safely.</x:v>
+        <x:v>Success, failure and pending states are handled safely in sandbox. Refund lifecycle remains excluded by V1-004.</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented in sandbox</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
@@ -2269,7 +2269,7 @@
         <x:v>Reports reconcile to source records and export if required.</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
@@ -2333,7 +2333,7 @@
         <x:v>AI suggestions are labelled, Coach-reviewed before delivery to Member and never silently replace Coach judgment.</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -2365,7 +2365,7 @@
         <x:v>A restore test produces a recorded result and identified recovery time.</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="96" customHeight="1">
@@ -2407,7 +2407,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce9058c1b8846f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ba9c1a5caff48f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2747,7 +2747,7 @@
         <x:v>Backend + Finance</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
-        <x:v>Version 1 payments</x:v>
+        <x:v>PROD-012 live gateway</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
         <x:v>Must</x:v>
@@ -2853,6 +2853,38 @@
       </x:c>
       <x:c r="J15" s="30" t="str">
         <x:v>Proposed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="26" t="str">
+        <x:v>PROD-012</x:v>
+      </x:c>
+      <x:c r="B16" s="26" t="str">
+        <x:v>FR-010, NFR-005</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="str">
+        <x:v>System enables approved live payment gateways after production readiness approval.</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="str">
+        <x:v>Provider merchant credentials, signed live webhooks, idempotency, monitoring and settlement reconciliation</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="str">
+        <x:v>Backend + Finance + DevOps</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str">
+        <x:v>V1-003 sandbox payments, PROD-003 observability, security review</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="str">
+        <x:v>Live callbacks are signature-verified and idempotent; paid, pending and failed states reconcile to the provider without exposing credentials.</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="str">
+        <x:v>Planned</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2862,7 +2894,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890ae0d2473f48f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10c338de792f46b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(requirements): define email-only verification
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R51ef286399a64523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R7c6fca849c3648b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rbbfea0165c25438b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R1f100769d17f4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rd9a28723c1d44eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R51dac861cfb44010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rf7f2dceee075459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rcb118a28f6ca4c8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1148,6 +1148,32 @@
         <x:v>Proposed</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="26" t="str">
+        <x:v>FR-016</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Account verification</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>Member</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>New member accounts are verified by a six-digit code delivered only by email. Phone or SMS verification is out of scope.</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>Version 1</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Only a verified sender domain may send the code. A valid email code changes registration to pending Receptionist approval; a phone number is not an authentication factor.</x:v>
+      </x:c>
+      <x:c r="H25" s="26" t="str">
+        <x:v>Updated</x:v>
+      </x:c>
+    </x:row>
     <x:row r="28">
       <x:c r="A28" s="25" t="str">
         <x:v>Role and permission summary</x:v>
@@ -1463,9 +1489,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c426c206d874e83"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2394fb5ba95414b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb9a6ed3716249b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875389986ac44b81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1267b21a952e4762"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R272888e6197842a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1946,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb3f01d9e2c4923"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4137e6681ef43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2407,7 +2433,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ba9c1a5caff48f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R318a53e276174c61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2894,7 +2920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10c338de792f46b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ba15171abbe403b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(payments): remove vnpay flow
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rd9a28723c1d44eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R51dac861cfb44010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rf7f2dceee075459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rcb118a28f6ca4c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R4a69d1cb9d8f4db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="R19f861d5a3554951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="Rc74236aae3c444b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R0991f78b626e4755"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -873,7 +873,7 @@
         <x:v>Manager, Receptionist, Member</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
-        <x:v>The system records manual or simulated payments and transaction status for memberships.</x:v>
+        <x:v>The system records cash, bank-transfer reconciliation and PayOS online payments for memberships.</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
         <x:v>Must</x:v>
@@ -882,10 +882,10 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
-        <x:v>Each payment has amount, method, payer, membership, paid timestamp and immutable transaction history. Only a successful payment activates a membership.</x:v>
+        <x:v>Each payment has amount, method, payer, membership, paid timestamp and immutable transaction history. Only a successful PayOS webhook or Receptionist-verified cash/bank-transfer payment activates a membership. VNPAY is out of scope.</x:v>
       </x:c>
       <x:c r="H14" s="19" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -1489,9 +1489,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875389986ac44b81"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1267b21a952e4762"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R272888e6197842a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e1dbd608dd44950"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb48bc576d454bf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef3797b3cfe43ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1946,7 +1946,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4137e6681ef43a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raebbdf28ec104f4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2433,7 +2433,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R318a53e276174c61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2cf65f04d7c455c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2920,7 +2920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ba15171abbe403b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83ed7ed26c6b4f04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: email member account credentials
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R378494ada49048d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rdb00d598bc284afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R823dbf5b123540dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R9f03ea7416f94165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update" sheetId="5" r:id="Re00af32f3b944f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rf58ef5f8f8ec42e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rf263207b2f91426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R528b81d4f35144ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rafb9077db7ae468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update" sheetId="5" r:id="R16ccc9525253458d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -873,7 +873,7 @@
         <x:v>Manager, Receptionist</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
-        <x:v>Staff can create and maintain member profiles.</x:v>
+        <x:v>Staff can create and maintain member profiles, and may create a member login account.</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
         <x:v>Must</x:v>
@@ -882,7 +882,7 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>Required fields are validated and duplicate member records are prevented.</x:v>
+        <x:v>Required fields are validated and duplicate member records are prevented. When creating a login account, email is required; a one-time temporary password is emailed and is returned only if delivery fails.</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
         <x:v>Completed</x:v>
@@ -1671,9 +1671,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b47a2f5815a45b2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ff1b71fa5724250"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06a2d5bc3df34327"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1393c658c7aa4238"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544ae6beb98f4c80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b513f72e1f452d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2128,7 +2128,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf302e5d1ffaf4f08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7142c21c084045"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2615,7 +2615,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38344e56e08c482d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dd23542f05c4c06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3102,7 +3102,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R015e7b5c79b941d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bf087134bf4a4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3478,7 +3478,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c2585ca31741ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0c201d86b94fb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: improve workspace feedback and facility queue performance
</commit_message>
<xml_diff>
--- a/backend/docs/sports-center-requirements.xlsx
+++ b/backend/docs/sports-center-requirements.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="Rf58ef5f8f8ec42e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Rf263207b2f91426c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R528b81d4f35144ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="Rafb9077db7ae468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update" sheetId="5" r:id="R16ccc9525253458d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Requirements" sheetId="1" r:id="R9c73c718bf9b420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP" sheetId="2" r:id="Re64ca36b41474ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version 1" sheetId="3" r:id="R92ac1fabbc164f8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="4" r:id="R9a0d7ef53cf04c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update" sheetId="5" r:id="Rc4de6d14bdf24d80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="12">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -85,8 +85,19 @@
       <x:color rgb="FF166534"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF263238"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF9A3412"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -106,6 +117,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF173D68"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EDF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -238,7 +254,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -387,6 +403,26 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1356,6 +1392,32 @@
         <x:v>Implemented - source verified</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="120" customHeight="1">
+      <x:c r="A27" s="63" t="str">
+        <x:v>FR-018</x:v>
+      </x:c>
+      <x:c r="B27" s="63" t="str">
+        <x:v>Interaction feedback and validation</x:v>
+      </x:c>
+      <x:c r="C27" s="63" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="D27" s="63" t="str">
+        <x:v>User-initiated actions show a clear result on screen. Forms report invalid or missing fields during entry and retain server-side validation after submission.</x:v>
+      </x:c>
+      <x:c r="E27" s="63" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F27" s="63" t="str">
+        <x:v>Update</x:v>
+      </x:c>
+      <x:c r="G27" s="63" t="str">
+        <x:v>Completed changes and exports show confirmation, including after navigation. Invalid fields show inline guidance while typing. Failures explain the field, business rule, permission or connection issue. An unknown server error names the action and shows a request ID when available. Never expose only an HTTP code or internal traces. Background polling must not repeat alerts.</x:v>
+      </x:c>
+      <x:c r="H27" s="64" t="str">
+        <x:v>Partial - source verified; UAT pending</x:v>
+      </x:c>
+    </x:row>
     <x:row r="28">
       <x:c r="A28" s="25" t="str">
         <x:v>Role and permission summary</x:v>
@@ -1671,9 +1733,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1393c658c7aa4238"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544ae6beb98f4c80"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b513f72e1f452d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59fd177fb05c4d59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8a9e8df4afb4a3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d46ac52f6cc4766"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2128,7 +2190,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7142c21c084045"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R659b87e1b0f64364"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2615,7 +2677,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dd23542f05c4c06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc857b61e4d5c4d4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3102,7 +3164,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bf087134bf4a4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14557f9861df4cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3139,7 +3201,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="35" t="str">
-        <x:v>Post-production updates reconciled with the current source on 2026-09-24. Statuses labelled source verified require browser and production UAT for final operational acceptance.</x:v>
+        <x:v>Post-production updates. Existing rows were source-verified on 2026-09-24; feedback and validation requirements were added on 2026-09-27. Browser and production UAT are required for operational acceptance.</x:v>
       </x:c>
       <x:c r="B2" s="35"/>
       <x:c r="C2" s="35"/>
@@ -3471,6 +3533,70 @@
         <x:v>Implemented - source verified</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="122" customHeight="1">
+      <x:c r="A14" s="66" t="str">
+        <x:v>UPD-010</x:v>
+      </x:c>
+      <x:c r="B14" s="66" t="str">
+        <x:v>FR-018</x:v>
+      </x:c>
+      <x:c r="C14" s="66" t="str">
+        <x:v>Form validation</x:v>
+      </x:c>
+      <x:c r="D14" s="66" t="str">
+        <x:v>Validate input during entry</x:v>
+      </x:c>
+      <x:c r="E14" s="66" t="str">
+        <x:v>Show field-level feedback while users enter account, package, membership, booking, attendance and payment data. Keep backend field validation authoritative.</x:v>
+      </x:c>
+      <x:c r="F14" s="66" t="str">
+        <x:v>Frontend + Backend</x:v>
+      </x:c>
+      <x:c r="G14" s="66" t="str">
+        <x:v>Existing forms and API validation</x:v>
+      </x:c>
+      <x:c r="H14" s="66" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="I14" s="66" t="str">
+        <x:v>A touched invalid field shows a specific message before submit. Correcting it clears the message. Submit focuses or identifies remaining invalid fields; backend validation maps to the corresponding field and never silently fails.</x:v>
+      </x:c>
+      <x:c r="J14" s="67" t="str">
+        <x:v>Partial - source verified; UAT pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="140" customHeight="1">
+      <x:c r="A15" s="63" t="str">
+        <x:v>UPD-011</x:v>
+      </x:c>
+      <x:c r="B15" s="63" t="str">
+        <x:v>FR-018, NFR-003</x:v>
+      </x:c>
+      <x:c r="C15" s="63" t="str">
+        <x:v>Outcome feedback</x:v>
+      </x:c>
+      <x:c r="D15" s="63" t="str">
+        <x:v>Explain success and failure for user actions</x:v>
+      </x:c>
+      <x:c r="E15" s="63" t="str">
+        <x:v>Show persistent-on-navigation success/error feedback for user-triggered writes, authentication, exports and copy actions. Preserve safe backend domain errors, field details and request IDs.</x:v>
+      </x:c>
+      <x:c r="F15" s="63" t="str">
+        <x:v>Frontend + Backend</x:v>
+      </x:c>
+      <x:c r="G15" s="63" t="str">
+        <x:v>API error envelope and notification UI</x:v>
+      </x:c>
+      <x:c r="H15" s="63" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="I15" s="63" t="str">
+        <x:v>Each attempted action reports success or failure on screen. Permission failures explain that the account lacks the required function; business failures state the rule returned by the API. Unknown server failures identify the action and include a request ID when available, without showing raw HTTP codes, stack traces or invented causes. Automatic polling errors are visible without repeated toasts.</x:v>
+      </x:c>
+      <x:c r="J15" s="64" t="str">
+        <x:v>Partial - source verified; UAT pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -3478,7 +3604,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0c201d86b94fb6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea120ce360aa4a5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>